<commit_message>
PDF-solicitud de suelo con mapa de racks
</commit_message>
<xml_diff>
--- a/Program/Datos/datos_DCE.xlsx
+++ b/Program/Datos/datos_DCE.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mhoyosme\Desktop\Proyecto\Program\Datos\DB\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mhoyosme\Desktop\Proyecto\Program\Datos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEB32870-A2B8-49FF-A16F-935F70A8B45D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DA555F2-AC30-4F18-A5DD-A1907411CB37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TR" sheetId="1" r:id="rId1"/>
@@ -22,11 +22,137 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="55">
+  <si>
+    <t>rectificador_id</t>
+  </si>
   <si>
     <t>fecha</t>
   </si>
   <si>
+    <t>voltaje_ac_entrada</t>
+  </si>
+  <si>
+    <t>voltaje_dc_salida</t>
+  </si>
+  <si>
+    <t>corriente_dc_total</t>
+  </si>
+  <si>
+    <t>porcentaje_carga</t>
+  </si>
+  <si>
+    <t>modo_sistema</t>
+  </si>
+  <si>
+    <t>num_fases</t>
+  </si>
+  <si>
+    <t>modulos_instalados</t>
+  </si>
+  <si>
+    <t>modulos_fallados</t>
+  </si>
+  <si>
+    <t>corriente_baterias</t>
+  </si>
+  <si>
+    <t>temp_baterias</t>
+  </si>
+  <si>
+    <t>corriente_carga</t>
+  </si>
+  <si>
+    <t>Float</t>
+  </si>
+  <si>
+    <t>2026-02-23 09:45:02</t>
+  </si>
+  <si>
+    <t>2026-02-23 09:45:04</t>
+  </si>
+  <si>
+    <t>2026-02-23 09:53:32</t>
+  </si>
+  <si>
+    <t>2026-02-23 09:53:34</t>
+  </si>
+  <si>
+    <t>2026-03-03 09:44:59</t>
+  </si>
+  <si>
+    <t>2026-03-03 09:45:00</t>
+  </si>
+  <si>
+    <t>2026-03-10 15:45:54</t>
+  </si>
+  <si>
+    <t>2026-03-10 15:45:55</t>
+  </si>
+  <si>
+    <t>voltaje_ac_l1_l2</t>
+  </si>
+  <si>
+    <t>voltaje_ac_l2_l3</t>
+  </si>
+  <si>
+    <t>voltaje_ac_l3_l1</t>
+  </si>
+  <si>
+    <t>frecuencia_sistema</t>
+  </si>
+  <si>
+    <t>voltaje_bateria</t>
+  </si>
+  <si>
+    <t>voltaje_gen_l1_l2</t>
+  </si>
+  <si>
+    <t>voltaje_gen_l2_l3</t>
+  </si>
+  <si>
+    <t>voltaje_gen_l3_l1</t>
+  </si>
+  <si>
+    <t>frecuencia_gen</t>
+  </si>
+  <si>
+    <t>rpm_gen</t>
+  </si>
+  <si>
+    <t>corriente_ac_l1</t>
+  </si>
+  <si>
+    <t>corriente_ac_l2</t>
+  </si>
+  <si>
+    <t>corriente_ac_l3</t>
+  </si>
+  <si>
+    <t>potencia_activa_kw</t>
+  </si>
+  <si>
+    <t>potencia_reactiva_kvar</t>
+  </si>
+  <si>
+    <t>potencia_aparente_kva</t>
+  </si>
+  <si>
+    <t>factor_potencia</t>
+  </si>
+  <si>
+    <t>2026-02-23 09:44:59</t>
+  </si>
+  <si>
+    <t>2026-02-23 09:53:29</t>
+  </si>
+  <si>
+    <t>2026-03-03 09:44:56</t>
+  </si>
+  <si>
+    <t>2026-03-10 15:45:50</t>
+  </si>
+  <si>
     <t>corriente_ac_r</t>
   </si>
   <si>
@@ -60,121 +186,7 @@
     <t>2026-03-03 09:44:57</t>
   </si>
   <si>
-    <t>voltaje_ac_l1_l2</t>
-  </si>
-  <si>
-    <t>voltaje_ac_l2_l3</t>
-  </si>
-  <si>
-    <t>voltaje_ac_l3_l1</t>
-  </si>
-  <si>
-    <t>frecuencia_sistema</t>
-  </si>
-  <si>
-    <t>voltaje_bateria</t>
-  </si>
-  <si>
-    <t>voltaje_gen_l1_l2</t>
-  </si>
-  <si>
-    <t>voltaje_gen_l2_l3</t>
-  </si>
-  <si>
-    <t>voltaje_gen_l3_l1</t>
-  </si>
-  <si>
-    <t>frecuencia_gen</t>
-  </si>
-  <si>
-    <t>rpm_gen</t>
-  </si>
-  <si>
-    <t>corriente_ac_l1</t>
-  </si>
-  <si>
-    <t>corriente_ac_l2</t>
-  </si>
-  <si>
-    <t>corriente_ac_l3</t>
-  </si>
-  <si>
-    <t>potencia_activa_kw</t>
-  </si>
-  <si>
-    <t>potencia_reactiva_kvar</t>
-  </si>
-  <si>
-    <t>potencia_aparente_kva</t>
-  </si>
-  <si>
-    <t>factor_potencia</t>
-  </si>
-  <si>
-    <t>2026-02-23 09:44:59</t>
-  </si>
-  <si>
-    <t>2026-02-23 09:53:29</t>
-  </si>
-  <si>
-    <t>2026-03-03 09:44:56</t>
-  </si>
-  <si>
-    <t>rectificador_id</t>
-  </si>
-  <si>
-    <t>voltaje_ac_entrada</t>
-  </si>
-  <si>
-    <t>voltaje_dc_salida</t>
-  </si>
-  <si>
-    <t>corriente_dc_total</t>
-  </si>
-  <si>
-    <t>porcentaje_carga</t>
-  </si>
-  <si>
-    <t>modo_sistema</t>
-  </si>
-  <si>
-    <t>num_fases</t>
-  </si>
-  <si>
-    <t>modulos_instalados</t>
-  </si>
-  <si>
-    <t>modulos_fallados</t>
-  </si>
-  <si>
-    <t>corriente_baterias</t>
-  </si>
-  <si>
-    <t>temp_baterias</t>
-  </si>
-  <si>
-    <t>corriente_carga</t>
-  </si>
-  <si>
-    <t>Float</t>
-  </si>
-  <si>
-    <t>2026-02-23 09:45:02</t>
-  </si>
-  <si>
-    <t>2026-02-23 09:45:04</t>
-  </si>
-  <si>
-    <t>2026-02-23 09:53:32</t>
-  </si>
-  <si>
-    <t>2026-02-23 09:53:34</t>
-  </si>
-  <si>
-    <t>2026-03-03 09:44:59</t>
-  </si>
-  <si>
-    <t>2026-03-03 09:45:00</t>
+    <t>2026-03-10 15:45:52</t>
   </si>
 </sst>
 </file>
@@ -235,10 +247,10 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -573,74 +585,74 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R5"/>
+  <dimension ref="A1:Y6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="29.140625" customWidth="1"/>
-    <col min="2" max="2" width="21" customWidth="1"/>
-    <col min="3" max="3" width="16.140625" customWidth="1"/>
-    <col min="4" max="4" width="19" customWidth="1"/>
-    <col min="18" max="18" width="23.85546875" customWidth="1"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="L1" s="1" t="s">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A2" s="2">
+      <c r="I1" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="S1" s="2"/>
+      <c r="T1" s="2"/>
+      <c r="U1" s="2"/>
+      <c r="V1" s="2"/>
+      <c r="W1" s="2"/>
+      <c r="X1" s="2"/>
+      <c r="Y1" s="2"/>
+    </row>
+    <row r="2" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A2" s="1">
         <v>45993.645833333343</v>
       </c>
       <c r="B2">
@@ -695,9 +707,9 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="B3">
         <v>214</v>
@@ -751,9 +763,9 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="B4">
         <v>211</v>
@@ -807,9 +819,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="B5">
         <v>214</v>
@@ -860,6 +872,62 @@
         <v>22</v>
       </c>
       <c r="R5">
+        <v>0.98</v>
+      </c>
+    </row>
+    <row r="6" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6">
+        <v>212</v>
+      </c>
+      <c r="C6">
+        <v>214</v>
+      </c>
+      <c r="D6">
+        <v>214</v>
+      </c>
+      <c r="E6">
+        <v>60</v>
+      </c>
+      <c r="F6">
+        <v>27.5</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+      <c r="L6">
+        <v>60</v>
+      </c>
+      <c r="M6">
+        <v>58</v>
+      </c>
+      <c r="N6">
+        <v>59</v>
+      </c>
+      <c r="O6">
+        <v>21</v>
+      </c>
+      <c r="P6">
+        <v>-4</v>
+      </c>
+      <c r="Q6">
+        <v>22</v>
+      </c>
+      <c r="R6">
         <v>0.98</v>
       </c>
     </row>
@@ -870,51 +938,47 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.140625" customWidth="1"/>
-    <col min="2" max="2" width="18.5703125" customWidth="1"/>
-    <col min="3" max="3" width="18.42578125" customWidth="1"/>
-    <col min="4" max="4" width="16.7109375" customWidth="1"/>
-    <col min="5" max="5" width="18.7109375" customWidth="1"/>
-    <col min="6" max="6" width="11.42578125" customWidth="1"/>
-    <col min="7" max="7" width="15.42578125" customWidth="1"/>
-    <col min="9" max="9" width="20.7109375" customWidth="1"/>
-    <col min="10" max="10" width="19.28515625" customWidth="1"/>
+    <col min="10" max="10" width="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="2">
+      <c r="B1" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
+      <c r="M1" s="2"/>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A2" s="1">
         <v>45993.645833333343</v>
       </c>
       <c r="B2">
@@ -942,9 +1006,9 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>51</v>
       </c>
       <c r="B3">
         <v>60.4</v>
@@ -971,9 +1035,9 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>52</v>
       </c>
       <c r="B4">
         <v>61.15</v>
@@ -1000,9 +1064,9 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>53</v>
       </c>
       <c r="B5">
         <v>57.27</v>
@@ -1027,6 +1091,35 @@
       </c>
       <c r="I5">
         <v>22.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B6">
+        <v>70.989999999999995</v>
+      </c>
+      <c r="C6">
+        <v>72.14</v>
+      </c>
+      <c r="D6">
+        <v>74.25</v>
+      </c>
+      <c r="E6">
+        <v>214.04</v>
+      </c>
+      <c r="F6">
+        <v>213.3</v>
+      </c>
+      <c r="G6">
+        <v>218.61</v>
+      </c>
+      <c r="H6">
+        <v>23</v>
+      </c>
+      <c r="I6">
+        <v>21.5</v>
       </c>
     </row>
   </sheetData>
@@ -1036,59 +1129,61 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:O11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="20.42578125" customWidth="1"/>
-    <col min="13" max="13" width="22" customWidth="1"/>
+    <col min="12" max="12" width="13.42578125" customWidth="1"/>
+    <col min="13" max="13" width="21.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="2"/>
+      <c r="O1" s="2"/>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="1">
         <v>45985.416666666657</v>
       </c>
       <c r="C2">
@@ -1104,7 +1199,7 @@
         <v>10</v>
       </c>
       <c r="G2" t="s">
-        <v>44</v>
+        <v>13</v>
       </c>
       <c r="H2">
         <v>3</v>
@@ -1125,11 +1220,11 @@
         <v>119</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="1">
         <v>45986.416666608799</v>
       </c>
       <c r="C3">
@@ -1145,7 +1240,7 @@
         <v>14</v>
       </c>
       <c r="G3" t="s">
-        <v>44</v>
+        <v>13</v>
       </c>
       <c r="H3">
         <v>3</v>
@@ -1166,12 +1261,12 @@
         <v>157</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>45</v>
+        <v>14</v>
       </c>
       <c r="C4">
         <v>214</v>
@@ -1207,12 +1302,12 @@
         <v>123</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>46</v>
+        <v>15</v>
       </c>
       <c r="C5">
         <v>214</v>
@@ -1248,12 +1343,12 @@
         <v>159</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>47</v>
+        <v>16</v>
       </c>
       <c r="C6">
         <v>211</v>
@@ -1268,7 +1363,7 @@
         <v>10</v>
       </c>
       <c r="G6" t="s">
-        <v>44</v>
+        <v>13</v>
       </c>
       <c r="H6">
         <v>3</v>
@@ -1289,12 +1384,12 @@
         <v>119</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2</v>
       </c>
       <c r="B7" t="s">
-        <v>48</v>
+        <v>17</v>
       </c>
       <c r="C7">
         <v>211</v>
@@ -1309,7 +1404,7 @@
         <v>15</v>
       </c>
       <c r="G7" t="s">
-        <v>44</v>
+        <v>13</v>
       </c>
       <c r="H7">
         <v>3</v>
@@ -1330,12 +1425,12 @@
         <v>159</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>1</v>
       </c>
       <c r="B8" t="s">
-        <v>49</v>
+        <v>18</v>
       </c>
       <c r="C8">
         <v>215</v>
@@ -1350,7 +1445,7 @@
         <v>10</v>
       </c>
       <c r="G8" t="s">
-        <v>44</v>
+        <v>13</v>
       </c>
       <c r="H8">
         <v>3</v>
@@ -1371,12 +1466,12 @@
         <v>118</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2</v>
       </c>
       <c r="B9" t="s">
-        <v>50</v>
+        <v>19</v>
       </c>
       <c r="C9">
         <v>215</v>
@@ -1391,7 +1486,7 @@
         <v>14</v>
       </c>
       <c r="G9" t="s">
-        <v>44</v>
+        <v>13</v>
       </c>
       <c r="H9">
         <v>3</v>
@@ -1409,6 +1504,88 @@
         <v>27</v>
       </c>
       <c r="M9">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>1</v>
+      </c>
+      <c r="B10" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10">
+        <v>214</v>
+      </c>
+      <c r="D10">
+        <v>54.55</v>
+      </c>
+      <c r="E10">
+        <v>118</v>
+      </c>
+      <c r="F10">
+        <v>10</v>
+      </c>
+      <c r="G10" t="s">
+        <v>13</v>
+      </c>
+      <c r="H10">
+        <v>3</v>
+      </c>
+      <c r="I10">
+        <v>21</v>
+      </c>
+      <c r="J10">
+        <v>0</v>
+      </c>
+      <c r="K10">
+        <v>0</v>
+      </c>
+      <c r="L10">
+        <v>30</v>
+      </c>
+      <c r="M10">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>2</v>
+      </c>
+      <c r="B11" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11">
+        <v>213</v>
+      </c>
+      <c r="D11">
+        <v>54.55</v>
+      </c>
+      <c r="E11">
+        <v>157</v>
+      </c>
+      <c r="F11">
+        <v>14</v>
+      </c>
+      <c r="G11" t="s">
+        <v>13</v>
+      </c>
+      <c r="H11">
+        <v>3</v>
+      </c>
+      <c r="I11">
+        <v>19</v>
+      </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
+      <c r="K11">
+        <v>0</v>
+      </c>
+      <c r="L11">
+        <v>29</v>
+      </c>
+      <c r="M11">
         <v>157</v>
       </c>
     </row>

</xml_diff>